<commit_message>
Siliconomics v0.6.1：液冷（M19、Rack 頁 D 節、液冷份額表 K6-lc；CF04、CF12）
- 橋接表 cool、avc 的分歧管／內容調整／滲透率／份額相對值、jentech 冷板元件份額移入本庫；橋接表、avc、auras、jentech 改讀（數值不變）
- CF12：市場定義為機架內液冷＋分歧管，台達電屬機架外，不入份額表

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V11Bd11jZKXZ5hH5AjB7NJ
</commit_message>
<xml_diff>
--- a/auras/dist/20261025_雙鴻模型_v0.1.1.xlsx
+++ b/auras/dist/20261025_雙鴻模型_v0.1.1.xlsx
@@ -6588,26 +6588,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">avc/dist/20261025_</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">奇鋐模型</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">_v0.2.1.xlsx</t>
+      <t xml:space="preserve">siliconomics</t>
     </r>
     <r>
       <rPr>
@@ -6626,18 +6607,28 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">In!D28:F28</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">奇鋐模型的假設（唯讀）；雙鴻另做機架分歧管（</t>
+      <t xml:space="preserve">SIF_lc_mani</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Siliconomics M19</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（與奇鋐模型同一值）；雙鴻另做機架分歧管（</t>
     </r>
     <r>
       <rPr>
@@ -6834,26 +6825,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">avc/dist/20261025_</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">奇鋐模型</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">_v0.2.1.xlsx</t>
+      <t xml:space="preserve">siliconomics</t>
     </r>
     <r>
       <rPr>
@@ -6872,18 +6844,28 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">In!D29:F29</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">奇鋐模型的假設（唯讀）：</t>
+      <t xml:space="preserve">SIF_lc_adj_27</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Siliconomics M19</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（與奇鋐模型同一值）：</t>
     </r>
     <r>
       <rPr>
@@ -7090,26 +7072,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">avc/dist/20261025_</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">奇鋐模型</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">_v0.2.1.xlsx</t>
+      <t xml:space="preserve">siliconomics</t>
     </r>
     <r>
       <rPr>
@@ -7128,7 +7091,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">In!D30:F30</t>
+      <t xml:space="preserve">SIF_lc_adj_28</t>
     </r>
   </si>
   <si>
@@ -7268,26 +7231,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">avc/dist/20261025_</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">奇鋐模型</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">_v0.2.1.xlsx</t>
+      <t xml:space="preserve">siliconomics</t>
     </r>
     <r>
       <rPr>
@@ -7306,7 +7250,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">In!D31:F31</t>
+      <t xml:space="preserve">SIF_lc_adj_29</t>
     </r>
   </si>
   <si>
@@ -7370,26 +7314,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">avc/dist/20261025_</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">奇鋐模型</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">_v0.2.1.xlsx</t>
+      <t xml:space="preserve">siliconomics</t>
     </r>
     <r>
       <rPr>
@@ -7408,18 +7333,28 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">In!D32:F32</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">奇鋐模型的假設（唯讀；</t>
+      <t xml:space="preserve">SIF_lc_pen_26</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Siliconomics M19</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（與奇鋐模型同一值；</t>
     </r>
     <r>
       <rPr>
@@ -7654,26 +7589,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">avc/dist/20261025_</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">奇鋐模型</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">_v0.2.1.xlsx</t>
+      <t xml:space="preserve">siliconomics</t>
     </r>
     <r>
       <rPr>
@@ -7692,7 +7608,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">In!D33:F33</t>
+      <t xml:space="preserve">SIF_lc_pen_27</t>
     </r>
   </si>
   <si>
@@ -7756,26 +7672,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">avc/dist/20261025_</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">奇鋐模型</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">_v0.2.1.xlsx</t>
+      <t xml:space="preserve">siliconomics</t>
     </r>
     <r>
       <rPr>
@@ -7794,7 +7691,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">In!D34:F34</t>
+      <t xml:space="preserve">SIF_lc_pen_28</t>
     </r>
   </si>
   <si>
@@ -7858,26 +7755,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">avc/dist/20261025_</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">奇鋐模型</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">_v0.2.1.xlsx</t>
+      <t xml:space="preserve">siliconomics</t>
     </r>
     <r>
       <rPr>
@@ -7896,7 +7774,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">In!D35:F35</t>
+      <t xml:space="preserve">SIF_lc_pen_29</t>
     </r>
   </si>
   <si>
@@ -7941,26 +7819,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">avc/dist/20261025_</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">奇鋐模型</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">_v0.2.1.xlsx</t>
+      <t xml:space="preserve">siliconomics</t>
     </r>
     <r>
       <rPr>
@@ -7979,7 +7838,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">In!D36:F36</t>
+      <t xml:space="preserve">SIF_lc_avrel_27</t>
     </r>
     <r>
       <rPr>
@@ -8215,26 +8074,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">avc/dist/20261025_</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">奇鋐模型</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">_v0.2.1.xlsx</t>
+      <t xml:space="preserve">siliconomics</t>
     </r>
     <r>
       <rPr>
@@ -8253,7 +8093,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">In!D37:F37</t>
+      <t xml:space="preserve">SIF_lc_avrel_28</t>
     </r>
     <r>
       <rPr>
@@ -8307,26 +8147,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">avc/dist/20261025_</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">奇鋐模型</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">_v0.2.1.xlsx</t>
+      <t xml:space="preserve">siliconomics</t>
     </r>
     <r>
       <rPr>
@@ -8345,7 +8166,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">In!D38:F38</t>
+      <t xml:space="preserve">SIF_lc_avrel_29</t>
     </r>
     <r>
       <rPr>
@@ -36699,7 +36520,7 @@
       <c r="H24" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="I24" s="3" t="s">
+      <c r="I24" s="7" t="s">
         <v>99</v>
       </c>
     </row>
@@ -36728,7 +36549,7 @@
       <c r="H25" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="I25" s="3" t="s">
+      <c r="I25" s="7" t="s">
         <v>103</v>
       </c>
     </row>
@@ -36815,7 +36636,7 @@
       <c r="H28" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="I28" s="3" t="s">
+      <c r="I28" s="7" t="s">
         <v>113</v>
       </c>
     </row>
@@ -38123,7 +37944,7 @@
         <v>50</v>
       </c>
       <c r="E81" s="6" t="n">
-        <v>0.498927641116676</v>
+        <v>0.498927641116677</v>
       </c>
       <c r="G81" s="7" t="s">
         <v>31</v>
@@ -38192,7 +38013,7 @@
         <v>50</v>
       </c>
       <c r="E84" s="6" t="n">
-        <v>0.424088494949175</v>
+        <v>0.424088494949176</v>
       </c>
       <c r="G84" s="7" t="s">
         <v>31</v>
@@ -39470,7 +39291,7 @@
       </c>
       <c r="C9" s="13" t="n">
         <f aca="false">avsh_26</f>
-        <v>0.498927641116676</v>
+        <v>0.498927641116677</v>
       </c>
       <c r="D9" s="13" t="n">
         <f aca="false">avsh_27</f>
@@ -39482,7 +39303,7 @@
       </c>
       <c r="F9" s="13" t="n">
         <f aca="false">avsh_29</f>
-        <v>0.424088494949175</v>
+        <v>0.424088494949176</v>
       </c>
       <c r="G9" s="3" t="s">
         <v>423</v>
@@ -39497,7 +39318,7 @@
       </c>
       <c r="C10" s="13" t="n">
         <f aca="false">C8+C9</f>
-        <v>0.657628417556846</v>
+        <v>0.657628417556847</v>
       </c>
       <c r="D10" s="13" t="n">
         <f aca="false">D8+D9</f>
@@ -39509,7 +39330,7 @@
       </c>
       <c r="F10" s="13" t="n">
         <f aca="false">F8+F9</f>
-        <v>0.558984154923319</v>
+        <v>0.55898415492332</v>
       </c>
       <c r="G10" s="3" t="s">
         <v>425</v>
@@ -39524,7 +39345,7 @@
       </c>
       <c r="C11" s="13" t="n">
         <f aca="false">1-C10</f>
-        <v>0.342371582443154</v>
+        <v>0.342371582443153</v>
       </c>
       <c r="D11" s="13" t="n">
         <f aca="false">1-D10</f>
@@ -39536,7 +39357,7 @@
       </c>
       <c r="F11" s="13" t="n">
         <f aca="false">1-F10</f>
-        <v>0.441015845076681</v>
+        <v>0.44101584507668</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -46319,15 +46140,15 @@
       </c>
       <c r="C19" s="13" t="n">
         <f aca="false">avsh_26+PL!D72</f>
-        <v>0.657628417556846</v>
+        <v>0.657628417556847</v>
       </c>
       <c r="E19" s="13" t="n">
         <f aca="false">avsh_26+PL!D110</f>
-        <v>0.657628417556846</v>
+        <v>0.657628417556847</v>
       </c>
       <c r="G19" s="13" t="n">
         <f aca="false">avsh_26+PL!D148</f>
-        <v>0.657628417556846</v>
+        <v>0.657628417556847</v>
       </c>
       <c r="I19" s="3" t="s">
         <v>687</v>
@@ -46388,15 +46209,15 @@
       </c>
       <c r="C22" s="13" t="n">
         <f aca="false">avsh_29+PL!G72</f>
-        <v>0.590724310211353</v>
+        <v>0.590724310211354</v>
       </c>
       <c r="E22" s="13" t="n">
         <f aca="false">avsh_29+PL!G110</f>
-        <v>0.558984154923319</v>
+        <v>0.55898415492332</v>
       </c>
       <c r="G22" s="13" t="n">
         <f aca="false">avsh_29+PL!G148</f>
-        <v>0.535179038457294</v>
+        <v>0.535179038457295</v>
       </c>
       <c r="I22" s="3" t="s">
         <v>687</v>

</xml_diff>